<commit_message>
fix: convert CRLF to LF in vendor
</commit_message>
<xml_diff>
--- a/vendor/x86/x86data/perfmon_data/TMA_Metrics.xlsx
+++ b/vendor/x86/x86data/perfmon_data/TMA_Metrics.xlsx
@@ -1,30 +1,3 @@
-
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahanna\Desktop\intel materials\TopDown\v3.5\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <bookViews>
-    <workbookView xWindow="2280" yWindow="810" windowWidth="16920" windowHeight="6210"/>
-  </bookViews>
-  <sheets>
-    <sheet name="public" sheetId="51" r:id="rId1"/>
-    <sheet name="Collateral" sheetId="2" r:id="rId2"/>
-    <sheet name="For tool developers" sheetId="6" r:id="rId3"/>
-    <sheet name="Revision History" sheetId="50" r:id="rId4"/>
-    <sheet name="Copyright" sheetId="9" r:id="rId5"/>
-  </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">public!$A$3:$V$130</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Revision History'!$B$26:$C$36</definedName>
-  </definedNames>
-  <calcPr calcId="152511"/>
-</workbook>
-</file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
@@ -9457,1101 +9430,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="11" customWidth="1"/>
-    <col min="3" max="3" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.28515625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="25" t="s">
-        <v>363</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" s="30" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="89" t="s">
-        <v>524</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" s="30" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C4" s="1" t="s">
-        <v>525</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>526</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>527</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" s="30" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B6" s="1" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C7" s="15" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B9" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C10" s="1" t="s">
-        <v>229</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>230</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="B6" r:id="rId1" display="Intel® Architecture Optimization Reference Manual, Top-Down Analysis Method chapter"/>
-    <hyperlink ref="C10" r:id="rId2" display="http://intelstudios.edgesuite.net/idf/2015/sf/aep/ARCS002/ARCS002.html"/>
-    <hyperlink ref="D10" r:id="rId3" display="http://www.intel.com/idfsessionsSF"/>
-    <hyperlink ref="C4" r:id="rId4" display="https://sites.google.com/site/analysismethods/yasin-pubs/TopDown-Yasin-ISPASS14.pdf?attredirects=0"/>
-    <hyperlink ref="D4" r:id="rId5" display="https://sites.google.com/site/analysismethods/yasin-pubs/TopDown-yasin-ISPASS14-foils.pdf?attredirects=0"/>
-    <hyperlink ref="E4" r:id="rId6" display="https://sites.google.com/site/analysismethods/yasin-pubs/TopDown-Yasin-ISPASS14-data.xlsx?attredirects=0"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId7"/>
-  <drawing r:id="rId8"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H44"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.85546875" customWidth="1"/>
-    <col min="4" max="4" width="16.140625" customWidth="1"/>
-    <col min="5" max="5" width="15.7109375" customWidth="1"/>
-    <col min="7" max="7" width="40.85546875" customWidth="1"/>
-    <col min="8" max="8" width="84.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="30" t="s">
-        <v>175</v>
-      </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="30"/>
-      <c r="B2" s="30" t="s">
-        <v>176</v>
-      </c>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="30"/>
-      <c r="B3" s="30"/>
-      <c r="C3" s="30" t="s">
-        <v>177</v>
-      </c>
-      <c r="D3" s="30" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="30"/>
-      <c r="B4" s="30" t="s">
-        <v>179</v>
-      </c>
-      <c r="C4" s="30" t="s">
-        <v>583</v>
-      </c>
-      <c r="D4" s="30"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="30"/>
-      <c r="B5" s="30" t="s">
-        <v>180</v>
-      </c>
-      <c r="C5" s="30" t="s">
-        <v>368</v>
-      </c>
-      <c r="D5" s="30"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="30"/>
-      <c r="B6" s="30" t="s">
-        <v>369</v>
-      </c>
-      <c r="C6" s="30" t="s">
-        <v>181</v>
-      </c>
-      <c r="D6" s="30"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="30"/>
-      <c r="B7" s="30" t="s">
-        <v>182</v>
-      </c>
-      <c r="C7" s="30"/>
-      <c r="D7" s="30"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="30"/>
-      <c r="B8" s="30"/>
-      <c r="C8" s="30" t="s">
-        <v>183</v>
-      </c>
-      <c r="D8" s="30"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="30"/>
-      <c r="B9" s="30"/>
-      <c r="C9" s="30" t="s">
-        <v>184</v>
-      </c>
-      <c r="D9" s="30"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="30"/>
-      <c r="B10" s="30"/>
-      <c r="C10" s="34" t="s">
-        <v>185</v>
-      </c>
-      <c r="D10" s="30"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="30"/>
-      <c r="B11" s="30" t="s">
-        <v>186</v>
-      </c>
-      <c r="C11" s="30"/>
-      <c r="D11" s="30"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="30"/>
-      <c r="B12" s="30"/>
-      <c r="C12" s="34" t="s">
-        <v>370</v>
-      </c>
-      <c r="D12" s="30"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="30"/>
-      <c r="B13" s="30"/>
-      <c r="C13" s="34" t="s">
-        <v>203</v>
-      </c>
-      <c r="D13" s="30"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="30"/>
-      <c r="B14" s="30"/>
-      <c r="C14" s="34" t="s">
-        <v>371</v>
-      </c>
-      <c r="D14" s="30"/>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="30"/>
-      <c r="B15" s="30"/>
-      <c r="C15" s="30" t="s">
-        <v>372</v>
-      </c>
-      <c r="D15" s="30"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="30"/>
-      <c r="B16" s="30"/>
-      <c r="C16" s="34" t="s">
-        <v>205</v>
-      </c>
-      <c r="D16" s="30"/>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="30"/>
-      <c r="B17" s="30" t="s">
-        <v>187</v>
-      </c>
-      <c r="C17" s="30"/>
-      <c r="D17" s="30"/>
-      <c r="E17" s="30"/>
-      <c r="F17" s="30"/>
-      <c r="G17" s="30"/>
-      <c r="H17" s="30"/>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="30"/>
-      <c r="B18" s="30"/>
-      <c r="C18" s="30" t="s">
-        <v>206</v>
-      </c>
-      <c r="D18" s="30"/>
-      <c r="E18" s="30"/>
-      <c r="F18" s="30"/>
-      <c r="G18" s="30"/>
-      <c r="H18" s="30"/>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="30"/>
-      <c r="B19" s="30"/>
-      <c r="C19" s="34" t="s">
-        <v>207</v>
-      </c>
-      <c r="D19" s="30"/>
-      <c r="E19" s="30"/>
-      <c r="F19" s="30"/>
-      <c r="G19" s="30"/>
-      <c r="H19" s="30"/>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="30"/>
-      <c r="B20" s="30"/>
-      <c r="C20" s="34" t="s">
-        <v>373</v>
-      </c>
-      <c r="D20" s="30"/>
-      <c r="E20" s="30"/>
-      <c r="F20" s="30"/>
-      <c r="G20" s="30"/>
-      <c r="H20" s="30"/>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="30"/>
-      <c r="B21" s="30"/>
-      <c r="C21" s="34" t="s">
-        <v>204</v>
-      </c>
-      <c r="D21" s="30"/>
-      <c r="E21" s="30"/>
-      <c r="F21" s="30"/>
-      <c r="G21" s="30"/>
-      <c r="H21" s="30"/>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="30"/>
-      <c r="B22" s="30" t="s">
-        <v>188</v>
-      </c>
-      <c r="C22" s="30"/>
-      <c r="D22" s="30"/>
-      <c r="E22" s="30"/>
-      <c r="F22" s="30"/>
-      <c r="G22" s="30"/>
-      <c r="H22" s="30"/>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" s="30"/>
-      <c r="B23" s="30"/>
-      <c r="C23" s="30" t="s">
-        <v>189</v>
-      </c>
-      <c r="D23" s="30"/>
-      <c r="E23" s="30"/>
-      <c r="F23" s="30"/>
-      <c r="G23" s="30"/>
-      <c r="H23" s="30"/>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" s="30"/>
-      <c r="B24" s="30"/>
-      <c r="C24" s="30" t="s">
-        <v>374</v>
-      </c>
-      <c r="D24" s="30"/>
-      <c r="E24" s="30"/>
-      <c r="F24" s="30"/>
-      <c r="G24" s="30"/>
-      <c r="H24" s="30"/>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A25" s="30"/>
-      <c r="B25" s="30"/>
-      <c r="C25" s="32" t="s">
-        <v>375</v>
-      </c>
-      <c r="D25" s="30"/>
-      <c r="E25" s="30"/>
-      <c r="F25" s="30"/>
-      <c r="G25" s="30"/>
-      <c r="H25" s="30"/>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" s="30"/>
-      <c r="B26" s="30"/>
-      <c r="C26" s="32" t="s">
-        <v>376</v>
-      </c>
-      <c r="D26" s="30"/>
-      <c r="E26" s="30"/>
-      <c r="F26" s="30"/>
-      <c r="G26" s="30"/>
-      <c r="H26" s="30"/>
-    </row>
-    <row r="27" spans="1:8" s="30" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C27" s="32" t="s">
-        <v>512</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A28" s="30" t="s">
-        <v>377</v>
-      </c>
-      <c r="B28" s="30"/>
-      <c r="C28" s="30"/>
-      <c r="D28" s="30"/>
-      <c r="E28" s="30"/>
-      <c r="F28" s="30"/>
-      <c r="G28" s="30"/>
-      <c r="H28" s="30"/>
-    </row>
-    <row r="29" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A29" s="30"/>
-      <c r="B29" s="30" t="s">
-        <v>13</v>
-      </c>
-      <c r="C29" s="37" t="s">
-        <v>13</v>
-      </c>
-      <c r="D29" s="40" t="s">
-        <v>378</v>
-      </c>
-      <c r="E29" s="40" t="s">
-        <v>379</v>
-      </c>
-      <c r="F29" s="40" t="s">
-        <v>380</v>
-      </c>
-      <c r="G29" s="37" t="s">
-        <v>381</v>
-      </c>
-      <c r="H29" s="37" t="s">
-        <v>382</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" s="30"/>
-      <c r="B30" s="30"/>
-      <c r="C30" s="41" t="s">
-        <v>19</v>
-      </c>
-      <c r="D30" s="37" t="s">
-        <v>383</v>
-      </c>
-      <c r="E30" s="42" t="s">
-        <v>210</v>
-      </c>
-      <c r="F30" s="37" t="s">
-        <v>354</v>
-      </c>
-      <c r="G30" s="38" t="s">
-        <v>384</v>
-      </c>
-      <c r="H30" s="38" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A31" s="30"/>
-      <c r="B31" s="30"/>
-      <c r="C31" s="41" t="s">
-        <v>299</v>
-      </c>
-      <c r="D31" s="37" t="s">
-        <v>383</v>
-      </c>
-      <c r="E31" s="42" t="s">
-        <v>210</v>
-      </c>
-      <c r="F31" s="37" t="s">
-        <v>354</v>
-      </c>
-      <c r="G31" s="38" t="s">
-        <v>386</v>
-      </c>
-      <c r="H31" s="38" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A32" s="30"/>
-      <c r="B32" s="30"/>
-      <c r="C32" s="41" t="s">
-        <v>27</v>
-      </c>
-      <c r="D32" s="37" t="s">
-        <v>383</v>
-      </c>
-      <c r="E32" s="42" t="s">
-        <v>210</v>
-      </c>
-      <c r="F32" s="37" t="s">
-        <v>387</v>
-      </c>
-      <c r="G32" s="39" t="s">
-        <v>388</v>
-      </c>
-      <c r="H32" s="39" t="s">
-        <v>339</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A33" s="30"/>
-      <c r="B33" s="30"/>
-      <c r="C33" s="41" t="s">
-        <v>356</v>
-      </c>
-      <c r="D33" s="37" t="s">
-        <v>383</v>
-      </c>
-      <c r="E33" s="42" t="s">
-        <v>210</v>
-      </c>
-      <c r="F33" s="37" t="s">
-        <v>387</v>
-      </c>
-      <c r="G33" s="39" t="s">
-        <v>389</v>
-      </c>
-      <c r="H33" s="37"/>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A34" s="30"/>
-      <c r="B34" s="30"/>
-      <c r="C34" s="37" t="s">
-        <v>358</v>
-      </c>
-      <c r="D34" s="37" t="s">
-        <v>390</v>
-      </c>
-      <c r="E34" s="37" t="s">
-        <v>391</v>
-      </c>
-      <c r="F34" s="37" t="s">
-        <v>387</v>
-      </c>
-      <c r="G34" s="39"/>
-      <c r="H34" s="37"/>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A35" s="30"/>
-      <c r="B35" s="30"/>
-      <c r="C35" s="37" t="s">
-        <v>357</v>
-      </c>
-      <c r="D35" s="37" t="s">
-        <v>390</v>
-      </c>
-      <c r="E35" s="37" t="s">
-        <v>392</v>
-      </c>
-      <c r="F35" s="37" t="s">
-        <v>387</v>
-      </c>
-      <c r="G35" s="37"/>
-      <c r="H35" s="37"/>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A36" s="33"/>
-      <c r="B36" s="33" t="s">
-        <v>15</v>
-      </c>
-      <c r="C36" s="33"/>
-      <c r="D36" s="33"/>
-      <c r="E36" s="33"/>
-      <c r="F36" s="33"/>
-      <c r="G36" s="33"/>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A37" s="33"/>
-      <c r="B37" s="33"/>
-      <c r="C37" s="31" t="s">
-        <v>393</v>
-      </c>
-      <c r="D37" s="33"/>
-      <c r="E37" s="33"/>
-      <c r="F37" s="33"/>
-      <c r="G37" s="33"/>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A38" s="33"/>
-      <c r="B38" s="33"/>
-      <c r="C38" s="31" t="s">
-        <v>394</v>
-      </c>
-      <c r="D38" s="33"/>
-      <c r="E38" s="33"/>
-      <c r="F38" s="33"/>
-      <c r="G38" s="33"/>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A39" s="30"/>
-      <c r="B39" s="30" t="s">
-        <v>395</v>
-      </c>
-      <c r="C39" s="36"/>
-      <c r="D39" s="30"/>
-      <c r="E39" s="30" t="s">
-        <v>396</v>
-      </c>
-      <c r="F39" s="30"/>
-      <c r="G39" s="30"/>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A40" s="30"/>
-      <c r="B40" s="30"/>
-      <c r="C40" s="36" t="s">
-        <v>397</v>
-      </c>
-      <c r="D40" s="35"/>
-      <c r="E40" s="35" t="s">
-        <v>398</v>
-      </c>
-      <c r="F40" s="30"/>
-      <c r="G40" s="30"/>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A41" s="30"/>
-      <c r="B41" s="30"/>
-      <c r="C41" s="35"/>
-      <c r="D41" s="35"/>
-      <c r="E41" s="35" t="s">
-        <v>399</v>
-      </c>
-      <c r="F41" s="30"/>
-      <c r="G41" s="30"/>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A42" s="32" t="s">
-        <v>400</v>
-      </c>
-      <c r="B42" s="32"/>
-      <c r="C42" s="32"/>
-      <c r="D42" s="32"/>
-      <c r="E42" s="32"/>
-      <c r="F42" s="32"/>
-      <c r="G42" s="32"/>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A43" s="32"/>
-      <c r="B43" s="32" t="s">
-        <v>401</v>
-      </c>
-      <c r="C43" s="32"/>
-      <c r="D43" s="32"/>
-      <c r="E43" s="32"/>
-      <c r="F43" s="32"/>
-      <c r="G43" s="32"/>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A44" s="32"/>
-      <c r="B44" s="32" t="s">
-        <v>584</v>
-      </c>
-      <c r="C44" s="32"/>
-      <c r="D44" s="32"/>
-      <c r="E44" s="32"/>
-      <c r="F44" s="32"/>
-      <c r="G44" s="32"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C74"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="6.42578125" style="30" customWidth="1"/>
-    <col min="2" max="2" width="85.28515625" style="30" customWidth="1"/>
-    <col min="3" max="3" width="7.28515625" style="30" customWidth="1"/>
-    <col min="4" max="16384" width="9.140625" style="30"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" ht="18" x14ac:dyDescent="0.4">
-      <c r="A1" s="90">
-        <v>3.01</v>
-      </c>
-      <c r="B1" s="91" t="s">
-        <v>528</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" ht="18" x14ac:dyDescent="0.4">
-      <c r="A2" s="92">
-        <v>3.02</v>
-      </c>
-      <c r="B2" s="93" t="s">
-        <v>529</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="94"/>
-      <c r="B3" s="95" t="s">
-        <v>530</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="94"/>
-      <c r="B4" s="96" t="s">
-        <v>531</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="94"/>
-      <c r="B5" s="96" t="s">
-        <v>532</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="94"/>
-      <c r="B6" s="96" t="s">
-        <v>533</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="94"/>
-      <c r="B7" s="95" t="s">
-        <v>534</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="94"/>
-      <c r="B8" s="96" t="s">
-        <v>535</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="94"/>
-      <c r="B9" s="96" t="s">
-        <v>536</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="94"/>
-      <c r="B10" s="96" t="s">
-        <v>537</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="94"/>
-      <c r="B11" s="96" t="s">
-        <v>538</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="94"/>
-      <c r="B12" s="95" t="s">
-        <v>539</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" ht="18" x14ac:dyDescent="0.4">
-      <c r="A13" s="97">
-        <v>3.1</v>
-      </c>
-      <c r="B13" s="97" t="s">
-        <v>540</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A14" s="98"/>
-      <c r="B14" s="99" t="s">
-        <v>541</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A15" s="98"/>
-      <c r="B15" s="99" t="s">
-        <v>542</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A16" s="98"/>
-      <c r="B16" s="100" t="s">
-        <v>543</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A17" s="98"/>
-      <c r="B17" s="100" t="s">
-        <v>544</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A18" s="98"/>
-      <c r="B18" s="100" t="s">
-        <v>545</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A19" s="98"/>
-      <c r="B19" s="100" t="s">
-        <v>546</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A20" s="98"/>
-      <c r="B20" s="100" t="s">
-        <v>547</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" ht="18" x14ac:dyDescent="0.4">
-      <c r="A21" s="101">
-        <v>3.14</v>
-      </c>
-      <c r="B21" s="102" t="s">
-        <v>548</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A22" s="103"/>
-      <c r="B22" s="99" t="s">
-        <v>549</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A23" s="103"/>
-      <c r="B23" s="99" t="s">
-        <v>542</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A24" s="103"/>
-      <c r="B24" s="100" t="s">
-        <v>550</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A25" s="103"/>
-      <c r="B25" s="100" t="s">
-        <v>551</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" ht="18" x14ac:dyDescent="0.4">
-      <c r="A26" s="104">
-        <v>3.2</v>
-      </c>
-      <c r="B26" s="104" t="s">
-        <v>552</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" s="105"/>
-      <c r="B27" s="106" t="s">
-        <v>553</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="105"/>
-      <c r="B28" s="107" t="s">
-        <v>554</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" s="105"/>
-      <c r="B29" s="106" t="s">
-        <v>555</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" s="105"/>
-      <c r="B30" s="107" t="s">
-        <v>556</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" s="105"/>
-      <c r="B31" s="106" t="s">
-        <v>557</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32" s="105"/>
-      <c r="B32" s="107" t="s">
-        <v>558</v>
-      </c>
-      <c r="C32" s="108"/>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33" s="105"/>
-      <c r="B33" s="106" t="s">
-        <v>559</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A34" s="105"/>
-      <c r="B34" s="107" t="s">
-        <v>560</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A35" s="105"/>
-      <c r="B35" s="107" t="s">
-        <v>561</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A36" s="105"/>
-      <c r="B36" s="107" t="s">
-        <v>562</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" ht="18" x14ac:dyDescent="0.4">
-      <c r="A37" s="109">
-        <v>3.3</v>
-      </c>
-      <c r="B37" s="109" t="s">
-        <v>570</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A38" s="110"/>
-      <c r="B38" s="106" t="s">
-        <v>553</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A39" s="110"/>
-      <c r="B39" s="112" t="s">
-        <v>571</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A40" s="110"/>
-      <c r="B40" s="111" t="s">
-        <v>563</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A41" s="110"/>
-      <c r="B41" s="106" t="s">
-        <v>555</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A42" s="110"/>
-      <c r="B42" s="107" t="s">
-        <v>564</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A43" s="110"/>
-      <c r="B43" s="107" t="s">
-        <v>565</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A44" s="110"/>
-      <c r="B44" s="106" t="s">
-        <v>557</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A45" s="110"/>
-      <c r="B45" s="107" t="s">
-        <v>686</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A46" s="110"/>
-      <c r="B46" s="106" t="s">
-        <v>559</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A47" s="110"/>
-      <c r="B47" s="107" t="s">
-        <v>566</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A48" s="110"/>
-      <c r="B48" s="107" t="s">
-        <v>567</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A49" s="110"/>
-      <c r="B49" s="107" t="s">
-        <v>568</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A50" s="110"/>
-      <c r="B50" s="107" t="s">
-        <v>569</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" ht="18" x14ac:dyDescent="0.4">
-      <c r="A51" s="113">
-        <v>3.4</v>
-      </c>
-      <c r="B51" s="113" t="s">
-        <v>572</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A52" s="114"/>
-      <c r="B52" s="106" t="s">
-        <v>553</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A53" s="114"/>
-      <c r="B53" s="107" t="s">
-        <v>573</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A54" s="114"/>
-      <c r="B54" s="106" t="s">
-        <v>557</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A55" s="114"/>
-      <c r="B55" s="116" t="s">
-        <v>574</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A56" s="114"/>
-      <c r="B56" s="107" t="s">
-        <v>575</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A57" s="114"/>
-      <c r="B57" s="107" t="s">
-        <v>576</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A58" s="114"/>
-      <c r="B58" s="107" t="s">
-        <v>577</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A59" s="114"/>
-      <c r="B59" s="107" t="s">
-        <v>578</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A60" s="114"/>
-      <c r="B60" s="106" t="s">
-        <v>579</v>
-      </c>
-    </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A61" s="115"/>
-      <c r="B61" s="107" t="s">
-        <v>580</v>
-      </c>
-    </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A62" s="114"/>
-      <c r="B62" s="107" t="s">
-        <v>581</v>
-      </c>
-    </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A63" s="114"/>
-      <c r="B63" s="107" t="s">
-        <v>582</v>
-      </c>
-    </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A64" s="117">
-        <v>3.5</v>
-      </c>
-      <c r="B64" s="118" t="s">
-        <v>586</v>
-      </c>
-    </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A65" s="117"/>
-      <c r="B65" s="119" t="s">
-        <v>587</v>
-      </c>
-    </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A66" s="117"/>
-      <c r="B66" s="111" t="s">
-        <v>588</v>
-      </c>
-    </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A67" s="117"/>
-      <c r="B67" s="106" t="s">
-        <v>557</v>
-      </c>
-    </row>
-    <row r="68" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A68" s="117"/>
-      <c r="B68" s="132" t="s">
-        <v>684</v>
-      </c>
-    </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A69" s="117"/>
-      <c r="B69" s="120" t="s">
-        <v>685</v>
-      </c>
-    </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A70" s="117"/>
-      <c r="B70" s="120" t="s">
-        <v>689</v>
-      </c>
-    </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A71" s="117"/>
-      <c r="B71" s="121" t="s">
-        <v>690</v>
-      </c>
-    </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A72" s="117"/>
-      <c r="B72" s="106" t="s">
-        <v>579</v>
-      </c>
-    </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A73" s="117"/>
-      <c r="B73" s="121" t="s">
-        <v>589</v>
-      </c>
-    </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A74" s="117"/>
-      <c r="B74" s="121" t="s">
-        <v>691</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:A35"/>

</xml_diff>

<commit_message>
fix: normalize line endings (CRLF → LF)
</commit_message>
<xml_diff>
--- a/vendor/x86/x86data/perfmon_data/TMA_Metrics.xlsx
+++ b/vendor/x86/x86data/perfmon_data/TMA_Metrics.xlsx
@@ -1,30 +1,3 @@
-
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahanna\Desktop\intel materials\TopDown\v3.5\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <bookViews>
-    <workbookView xWindow="2280" yWindow="810" windowWidth="16920" windowHeight="6210"/>
-  </bookViews>
-  <sheets>
-    <sheet name="public" sheetId="51" r:id="rId1"/>
-    <sheet name="Collateral" sheetId="2" r:id="rId2"/>
-    <sheet name="For tool developers" sheetId="6" r:id="rId3"/>
-    <sheet name="Revision History" sheetId="50" r:id="rId4"/>
-    <sheet name="Copyright" sheetId="9" r:id="rId5"/>
-  </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">public!$A$3:$V$130</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Revision History'!$B$26:$C$36</definedName>
-  </definedNames>
-  <calcPr calcId="152511"/>
-</workbook>
-</file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
@@ -9457,1101 +9430,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="11" customWidth="1"/>
-    <col min="3" max="3" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.28515625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="25" t="s">
-        <v>363</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" s="30" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="89" t="s">
-        <v>524</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" s="30" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C4" s="1" t="s">
-        <v>525</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>526</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>527</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" s="30" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B6" s="1" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C7" s="15" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B9" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C10" s="1" t="s">
-        <v>229</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>230</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="B6" r:id="rId1" display="Intel® Architecture Optimization Reference Manual, Top-Down Analysis Method chapter"/>
-    <hyperlink ref="C10" r:id="rId2" display="http://intelstudios.edgesuite.net/idf/2015/sf/aep/ARCS002/ARCS002.html"/>
-    <hyperlink ref="D10" r:id="rId3" display="http://www.intel.com/idfsessionsSF"/>
-    <hyperlink ref="C4" r:id="rId4" display="https://sites.google.com/site/analysismethods/yasin-pubs/TopDown-Yasin-ISPASS14.pdf?attredirects=0"/>
-    <hyperlink ref="D4" r:id="rId5" display="https://sites.google.com/site/analysismethods/yasin-pubs/TopDown-yasin-ISPASS14-foils.pdf?attredirects=0"/>
-    <hyperlink ref="E4" r:id="rId6" display="https://sites.google.com/site/analysismethods/yasin-pubs/TopDown-Yasin-ISPASS14-data.xlsx?attredirects=0"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId7"/>
-  <drawing r:id="rId8"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H44"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.85546875" customWidth="1"/>
-    <col min="4" max="4" width="16.140625" customWidth="1"/>
-    <col min="5" max="5" width="15.7109375" customWidth="1"/>
-    <col min="7" max="7" width="40.85546875" customWidth="1"/>
-    <col min="8" max="8" width="84.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="30" t="s">
-        <v>175</v>
-      </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="30"/>
-      <c r="B2" s="30" t="s">
-        <v>176</v>
-      </c>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="30"/>
-      <c r="B3" s="30"/>
-      <c r="C3" s="30" t="s">
-        <v>177</v>
-      </c>
-      <c r="D3" s="30" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="30"/>
-      <c r="B4" s="30" t="s">
-        <v>179</v>
-      </c>
-      <c r="C4" s="30" t="s">
-        <v>583</v>
-      </c>
-      <c r="D4" s="30"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="30"/>
-      <c r="B5" s="30" t="s">
-        <v>180</v>
-      </c>
-      <c r="C5" s="30" t="s">
-        <v>368</v>
-      </c>
-      <c r="D5" s="30"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="30"/>
-      <c r="B6" s="30" t="s">
-        <v>369</v>
-      </c>
-      <c r="C6" s="30" t="s">
-        <v>181</v>
-      </c>
-      <c r="D6" s="30"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="30"/>
-      <c r="B7" s="30" t="s">
-        <v>182</v>
-      </c>
-      <c r="C7" s="30"/>
-      <c r="D7" s="30"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="30"/>
-      <c r="B8" s="30"/>
-      <c r="C8" s="30" t="s">
-        <v>183</v>
-      </c>
-      <c r="D8" s="30"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="30"/>
-      <c r="B9" s="30"/>
-      <c r="C9" s="30" t="s">
-        <v>184</v>
-      </c>
-      <c r="D9" s="30"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="30"/>
-      <c r="B10" s="30"/>
-      <c r="C10" s="34" t="s">
-        <v>185</v>
-      </c>
-      <c r="D10" s="30"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="30"/>
-      <c r="B11" s="30" t="s">
-        <v>186</v>
-      </c>
-      <c r="C11" s="30"/>
-      <c r="D11" s="30"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="30"/>
-      <c r="B12" s="30"/>
-      <c r="C12" s="34" t="s">
-        <v>370</v>
-      </c>
-      <c r="D12" s="30"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="30"/>
-      <c r="B13" s="30"/>
-      <c r="C13" s="34" t="s">
-        <v>203</v>
-      </c>
-      <c r="D13" s="30"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="30"/>
-      <c r="B14" s="30"/>
-      <c r="C14" s="34" t="s">
-        <v>371</v>
-      </c>
-      <c r="D14" s="30"/>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="30"/>
-      <c r="B15" s="30"/>
-      <c r="C15" s="30" t="s">
-        <v>372</v>
-      </c>
-      <c r="D15" s="30"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="30"/>
-      <c r="B16" s="30"/>
-      <c r="C16" s="34" t="s">
-        <v>205</v>
-      </c>
-      <c r="D16" s="30"/>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="30"/>
-      <c r="B17" s="30" t="s">
-        <v>187</v>
-      </c>
-      <c r="C17" s="30"/>
-      <c r="D17" s="30"/>
-      <c r="E17" s="30"/>
-      <c r="F17" s="30"/>
-      <c r="G17" s="30"/>
-      <c r="H17" s="30"/>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="30"/>
-      <c r="B18" s="30"/>
-      <c r="C18" s="30" t="s">
-        <v>206</v>
-      </c>
-      <c r="D18" s="30"/>
-      <c r="E18" s="30"/>
-      <c r="F18" s="30"/>
-      <c r="G18" s="30"/>
-      <c r="H18" s="30"/>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="30"/>
-      <c r="B19" s="30"/>
-      <c r="C19" s="34" t="s">
-        <v>207</v>
-      </c>
-      <c r="D19" s="30"/>
-      <c r="E19" s="30"/>
-      <c r="F19" s="30"/>
-      <c r="G19" s="30"/>
-      <c r="H19" s="30"/>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="30"/>
-      <c r="B20" s="30"/>
-      <c r="C20" s="34" t="s">
-        <v>373</v>
-      </c>
-      <c r="D20" s="30"/>
-      <c r="E20" s="30"/>
-      <c r="F20" s="30"/>
-      <c r="G20" s="30"/>
-      <c r="H20" s="30"/>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="30"/>
-      <c r="B21" s="30"/>
-      <c r="C21" s="34" t="s">
-        <v>204</v>
-      </c>
-      <c r="D21" s="30"/>
-      <c r="E21" s="30"/>
-      <c r="F21" s="30"/>
-      <c r="G21" s="30"/>
-      <c r="H21" s="30"/>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="30"/>
-      <c r="B22" s="30" t="s">
-        <v>188</v>
-      </c>
-      <c r="C22" s="30"/>
-      <c r="D22" s="30"/>
-      <c r="E22" s="30"/>
-      <c r="F22" s="30"/>
-      <c r="G22" s="30"/>
-      <c r="H22" s="30"/>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" s="30"/>
-      <c r="B23" s="30"/>
-      <c r="C23" s="30" t="s">
-        <v>189</v>
-      </c>
-      <c r="D23" s="30"/>
-      <c r="E23" s="30"/>
-      <c r="F23" s="30"/>
-      <c r="G23" s="30"/>
-      <c r="H23" s="30"/>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" s="30"/>
-      <c r="B24" s="30"/>
-      <c r="C24" s="30" t="s">
-        <v>374</v>
-      </c>
-      <c r="D24" s="30"/>
-      <c r="E24" s="30"/>
-      <c r="F24" s="30"/>
-      <c r="G24" s="30"/>
-      <c r="H24" s="30"/>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A25" s="30"/>
-      <c r="B25" s="30"/>
-      <c r="C25" s="32" t="s">
-        <v>375</v>
-      </c>
-      <c r="D25" s="30"/>
-      <c r="E25" s="30"/>
-      <c r="F25" s="30"/>
-      <c r="G25" s="30"/>
-      <c r="H25" s="30"/>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" s="30"/>
-      <c r="B26" s="30"/>
-      <c r="C26" s="32" t="s">
-        <v>376</v>
-      </c>
-      <c r="D26" s="30"/>
-      <c r="E26" s="30"/>
-      <c r="F26" s="30"/>
-      <c r="G26" s="30"/>
-      <c r="H26" s="30"/>
-    </row>
-    <row r="27" spans="1:8" s="30" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="C27" s="32" t="s">
-        <v>512</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A28" s="30" t="s">
-        <v>377</v>
-      </c>
-      <c r="B28" s="30"/>
-      <c r="C28" s="30"/>
-      <c r="D28" s="30"/>
-      <c r="E28" s="30"/>
-      <c r="F28" s="30"/>
-      <c r="G28" s="30"/>
-      <c r="H28" s="30"/>
-    </row>
-    <row r="29" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A29" s="30"/>
-      <c r="B29" s="30" t="s">
-        <v>13</v>
-      </c>
-      <c r="C29" s="37" t="s">
-        <v>13</v>
-      </c>
-      <c r="D29" s="40" t="s">
-        <v>378</v>
-      </c>
-      <c r="E29" s="40" t="s">
-        <v>379</v>
-      </c>
-      <c r="F29" s="40" t="s">
-        <v>380</v>
-      </c>
-      <c r="G29" s="37" t="s">
-        <v>381</v>
-      </c>
-      <c r="H29" s="37" t="s">
-        <v>382</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" s="30"/>
-      <c r="B30" s="30"/>
-      <c r="C30" s="41" t="s">
-        <v>19</v>
-      </c>
-      <c r="D30" s="37" t="s">
-        <v>383</v>
-      </c>
-      <c r="E30" s="42" t="s">
-        <v>210</v>
-      </c>
-      <c r="F30" s="37" t="s">
-        <v>354</v>
-      </c>
-      <c r="G30" s="38" t="s">
-        <v>384</v>
-      </c>
-      <c r="H30" s="38" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A31" s="30"/>
-      <c r="B31" s="30"/>
-      <c r="C31" s="41" t="s">
-        <v>299</v>
-      </c>
-      <c r="D31" s="37" t="s">
-        <v>383</v>
-      </c>
-      <c r="E31" s="42" t="s">
-        <v>210</v>
-      </c>
-      <c r="F31" s="37" t="s">
-        <v>354</v>
-      </c>
-      <c r="G31" s="38" t="s">
-        <v>386</v>
-      </c>
-      <c r="H31" s="38" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A32" s="30"/>
-      <c r="B32" s="30"/>
-      <c r="C32" s="41" t="s">
-        <v>27</v>
-      </c>
-      <c r="D32" s="37" t="s">
-        <v>383</v>
-      </c>
-      <c r="E32" s="42" t="s">
-        <v>210</v>
-      </c>
-      <c r="F32" s="37" t="s">
-        <v>387</v>
-      </c>
-      <c r="G32" s="39" t="s">
-        <v>388</v>
-      </c>
-      <c r="H32" s="39" t="s">
-        <v>339</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A33" s="30"/>
-      <c r="B33" s="30"/>
-      <c r="C33" s="41" t="s">
-        <v>356</v>
-      </c>
-      <c r="D33" s="37" t="s">
-        <v>383</v>
-      </c>
-      <c r="E33" s="42" t="s">
-        <v>210</v>
-      </c>
-      <c r="F33" s="37" t="s">
-        <v>387</v>
-      </c>
-      <c r="G33" s="39" t="s">
-        <v>389</v>
-      </c>
-      <c r="H33" s="37"/>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A34" s="30"/>
-      <c r="B34" s="30"/>
-      <c r="C34" s="37" t="s">
-        <v>358</v>
-      </c>
-      <c r="D34" s="37" t="s">
-        <v>390</v>
-      </c>
-      <c r="E34" s="37" t="s">
-        <v>391</v>
-      </c>
-      <c r="F34" s="37" t="s">
-        <v>387</v>
-      </c>
-      <c r="G34" s="39"/>
-      <c r="H34" s="37"/>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A35" s="30"/>
-      <c r="B35" s="30"/>
-      <c r="C35" s="37" t="s">
-        <v>357</v>
-      </c>
-      <c r="D35" s="37" t="s">
-        <v>390</v>
-      </c>
-      <c r="E35" s="37" t="s">
-        <v>392</v>
-      </c>
-      <c r="F35" s="37" t="s">
-        <v>387</v>
-      </c>
-      <c r="G35" s="37"/>
-      <c r="H35" s="37"/>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A36" s="33"/>
-      <c r="B36" s="33" t="s">
-        <v>15</v>
-      </c>
-      <c r="C36" s="33"/>
-      <c r="D36" s="33"/>
-      <c r="E36" s="33"/>
-      <c r="F36" s="33"/>
-      <c r="G36" s="33"/>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A37" s="33"/>
-      <c r="B37" s="33"/>
-      <c r="C37" s="31" t="s">
-        <v>393</v>
-      </c>
-      <c r="D37" s="33"/>
-      <c r="E37" s="33"/>
-      <c r="F37" s="33"/>
-      <c r="G37" s="33"/>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A38" s="33"/>
-      <c r="B38" s="33"/>
-      <c r="C38" s="31" t="s">
-        <v>394</v>
-      </c>
-      <c r="D38" s="33"/>
-      <c r="E38" s="33"/>
-      <c r="F38" s="33"/>
-      <c r="G38" s="33"/>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A39" s="30"/>
-      <c r="B39" s="30" t="s">
-        <v>395</v>
-      </c>
-      <c r="C39" s="36"/>
-      <c r="D39" s="30"/>
-      <c r="E39" s="30" t="s">
-        <v>396</v>
-      </c>
-      <c r="F39" s="30"/>
-      <c r="G39" s="30"/>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A40" s="30"/>
-      <c r="B40" s="30"/>
-      <c r="C40" s="36" t="s">
-        <v>397</v>
-      </c>
-      <c r="D40" s="35"/>
-      <c r="E40" s="35" t="s">
-        <v>398</v>
-      </c>
-      <c r="F40" s="30"/>
-      <c r="G40" s="30"/>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A41" s="30"/>
-      <c r="B41" s="30"/>
-      <c r="C41" s="35"/>
-      <c r="D41" s="35"/>
-      <c r="E41" s="35" t="s">
-        <v>399</v>
-      </c>
-      <c r="F41" s="30"/>
-      <c r="G41" s="30"/>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A42" s="32" t="s">
-        <v>400</v>
-      </c>
-      <c r="B42" s="32"/>
-      <c r="C42" s="32"/>
-      <c r="D42" s="32"/>
-      <c r="E42" s="32"/>
-      <c r="F42" s="32"/>
-      <c r="G42" s="32"/>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A43" s="32"/>
-      <c r="B43" s="32" t="s">
-        <v>401</v>
-      </c>
-      <c r="C43" s="32"/>
-      <c r="D43" s="32"/>
-      <c r="E43" s="32"/>
-      <c r="F43" s="32"/>
-      <c r="G43" s="32"/>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A44" s="32"/>
-      <c r="B44" s="32" t="s">
-        <v>584</v>
-      </c>
-      <c r="C44" s="32"/>
-      <c r="D44" s="32"/>
-      <c r="E44" s="32"/>
-      <c r="F44" s="32"/>
-      <c r="G44" s="32"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C74"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="6.42578125" style="30" customWidth="1"/>
-    <col min="2" max="2" width="85.28515625" style="30" customWidth="1"/>
-    <col min="3" max="3" width="7.28515625" style="30" customWidth="1"/>
-    <col min="4" max="16384" width="9.140625" style="30"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" ht="18" x14ac:dyDescent="0.4">
-      <c r="A1" s="90">
-        <v>3.01</v>
-      </c>
-      <c r="B1" s="91" t="s">
-        <v>528</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" ht="18" x14ac:dyDescent="0.4">
-      <c r="A2" s="92">
-        <v>3.02</v>
-      </c>
-      <c r="B2" s="93" t="s">
-        <v>529</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="94"/>
-      <c r="B3" s="95" t="s">
-        <v>530</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="94"/>
-      <c r="B4" s="96" t="s">
-        <v>531</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="94"/>
-      <c r="B5" s="96" t="s">
-        <v>532</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="94"/>
-      <c r="B6" s="96" t="s">
-        <v>533</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="94"/>
-      <c r="B7" s="95" t="s">
-        <v>534</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="94"/>
-      <c r="B8" s="96" t="s">
-        <v>535</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="94"/>
-      <c r="B9" s="96" t="s">
-        <v>536</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="94"/>
-      <c r="B10" s="96" t="s">
-        <v>537</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="94"/>
-      <c r="B11" s="96" t="s">
-        <v>538</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="94"/>
-      <c r="B12" s="95" t="s">
-        <v>539</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" ht="18" x14ac:dyDescent="0.4">
-      <c r="A13" s="97">
-        <v>3.1</v>
-      </c>
-      <c r="B13" s="97" t="s">
-        <v>540</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A14" s="98"/>
-      <c r="B14" s="99" t="s">
-        <v>541</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A15" s="98"/>
-      <c r="B15" s="99" t="s">
-        <v>542</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A16" s="98"/>
-      <c r="B16" s="100" t="s">
-        <v>543</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A17" s="98"/>
-      <c r="B17" s="100" t="s">
-        <v>544</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A18" s="98"/>
-      <c r="B18" s="100" t="s">
-        <v>545</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A19" s="98"/>
-      <c r="B19" s="100" t="s">
-        <v>546</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A20" s="98"/>
-      <c r="B20" s="100" t="s">
-        <v>547</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" ht="18" x14ac:dyDescent="0.4">
-      <c r="A21" s="101">
-        <v>3.14</v>
-      </c>
-      <c r="B21" s="102" t="s">
-        <v>548</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A22" s="103"/>
-      <c r="B22" s="99" t="s">
-        <v>549</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A23" s="103"/>
-      <c r="B23" s="99" t="s">
-        <v>542</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A24" s="103"/>
-      <c r="B24" s="100" t="s">
-        <v>550</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A25" s="103"/>
-      <c r="B25" s="100" t="s">
-        <v>551</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" ht="18" x14ac:dyDescent="0.4">
-      <c r="A26" s="104">
-        <v>3.2</v>
-      </c>
-      <c r="B26" s="104" t="s">
-        <v>552</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" s="105"/>
-      <c r="B27" s="106" t="s">
-        <v>553</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="105"/>
-      <c r="B28" s="107" t="s">
-        <v>554</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" s="105"/>
-      <c r="B29" s="106" t="s">
-        <v>555</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" s="105"/>
-      <c r="B30" s="107" t="s">
-        <v>556</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" s="105"/>
-      <c r="B31" s="106" t="s">
-        <v>557</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32" s="105"/>
-      <c r="B32" s="107" t="s">
-        <v>558</v>
-      </c>
-      <c r="C32" s="108"/>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33" s="105"/>
-      <c r="B33" s="106" t="s">
-        <v>559</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A34" s="105"/>
-      <c r="B34" s="107" t="s">
-        <v>560</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A35" s="105"/>
-      <c r="B35" s="107" t="s">
-        <v>561</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A36" s="105"/>
-      <c r="B36" s="107" t="s">
-        <v>562</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" ht="18" x14ac:dyDescent="0.4">
-      <c r="A37" s="109">
-        <v>3.3</v>
-      </c>
-      <c r="B37" s="109" t="s">
-        <v>570</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A38" s="110"/>
-      <c r="B38" s="106" t="s">
-        <v>553</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A39" s="110"/>
-      <c r="B39" s="112" t="s">
-        <v>571</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A40" s="110"/>
-      <c r="B40" s="111" t="s">
-        <v>563</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A41" s="110"/>
-      <c r="B41" s="106" t="s">
-        <v>555</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A42" s="110"/>
-      <c r="B42" s="107" t="s">
-        <v>564</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A43" s="110"/>
-      <c r="B43" s="107" t="s">
-        <v>565</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A44" s="110"/>
-      <c r="B44" s="106" t="s">
-        <v>557</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A45" s="110"/>
-      <c r="B45" s="107" t="s">
-        <v>686</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A46" s="110"/>
-      <c r="B46" s="106" t="s">
-        <v>559</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A47" s="110"/>
-      <c r="B47" s="107" t="s">
-        <v>566</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A48" s="110"/>
-      <c r="B48" s="107" t="s">
-        <v>567</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A49" s="110"/>
-      <c r="B49" s="107" t="s">
-        <v>568</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A50" s="110"/>
-      <c r="B50" s="107" t="s">
-        <v>569</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" ht="18" x14ac:dyDescent="0.4">
-      <c r="A51" s="113">
-        <v>3.4</v>
-      </c>
-      <c r="B51" s="113" t="s">
-        <v>572</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A52" s="114"/>
-      <c r="B52" s="106" t="s">
-        <v>553</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A53" s="114"/>
-      <c r="B53" s="107" t="s">
-        <v>573</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A54" s="114"/>
-      <c r="B54" s="106" t="s">
-        <v>557</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A55" s="114"/>
-      <c r="B55" s="116" t="s">
-        <v>574</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A56" s="114"/>
-      <c r="B56" s="107" t="s">
-        <v>575</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A57" s="114"/>
-      <c r="B57" s="107" t="s">
-        <v>576</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A58" s="114"/>
-      <c r="B58" s="107" t="s">
-        <v>577</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A59" s="114"/>
-      <c r="B59" s="107" t="s">
-        <v>578</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A60" s="114"/>
-      <c r="B60" s="106" t="s">
-        <v>579</v>
-      </c>
-    </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A61" s="115"/>
-      <c r="B61" s="107" t="s">
-        <v>580</v>
-      </c>
-    </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A62" s="114"/>
-      <c r="B62" s="107" t="s">
-        <v>581</v>
-      </c>
-    </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A63" s="114"/>
-      <c r="B63" s="107" t="s">
-        <v>582</v>
-      </c>
-    </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A64" s="117">
-        <v>3.5</v>
-      </c>
-      <c r="B64" s="118" t="s">
-        <v>586</v>
-      </c>
-    </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A65" s="117"/>
-      <c r="B65" s="119" t="s">
-        <v>587</v>
-      </c>
-    </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A66" s="117"/>
-      <c r="B66" s="111" t="s">
-        <v>588</v>
-      </c>
-    </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A67" s="117"/>
-      <c r="B67" s="106" t="s">
-        <v>557</v>
-      </c>
-    </row>
-    <row r="68" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A68" s="117"/>
-      <c r="B68" s="132" t="s">
-        <v>684</v>
-      </c>
-    </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A69" s="117"/>
-      <c r="B69" s="120" t="s">
-        <v>685</v>
-      </c>
-    </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A70" s="117"/>
-      <c r="B70" s="120" t="s">
-        <v>689</v>
-      </c>
-    </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A71" s="117"/>
-      <c r="B71" s="121" t="s">
-        <v>690</v>
-      </c>
-    </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A72" s="117"/>
-      <c r="B72" s="106" t="s">
-        <v>579</v>
-      </c>
-    </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A73" s="117"/>
-      <c r="B73" s="121" t="s">
-        <v>589</v>
-      </c>
-    </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A74" s="117"/>
-      <c r="B74" s="121" t="s">
-        <v>691</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:A35"/>

</xml_diff>